<commit_message>
Update GAA results for 2026-03-04
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2003"/>
+  <dimension ref="A1:G2004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70919,6 +70919,43 @@
         </is>
       </c>
     </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Niall McInerney (Senior D) Cup</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>Ballyhaunis Community School</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr">
+        <is>
+          <t>Mount Sion CBS Post Primary</t>
+        </is>
+      </c>
+      <c r="D2004" t="inlineStr">
+        <is>
+          <t>04/03/2026</t>
+        </is>
+      </c>
+      <c r="E2004" t="inlineStr">
+        <is>
+          <t>UL Grounds</t>
+        </is>
+      </c>
+      <c r="F2004" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="G2004" t="inlineStr">
+        <is>
+          <t>7-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-07
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2004"/>
+  <dimension ref="A1:G2018"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70956,6 +70956,524 @@
         </is>
       </c>
     </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1A</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="D2005" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2005" t="inlineStr">
+        <is>
+          <t>Pearse Stadium</t>
+        </is>
+      </c>
+      <c r="F2005" t="inlineStr">
+        <is>
+          <t>0-35</t>
+        </is>
+      </c>
+      <c r="G2005" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1A</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2006" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2006" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2006" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+      <c r="G2006" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1B</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2007" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2007" t="inlineStr">
+        <is>
+          <t>Parnell Park</t>
+        </is>
+      </c>
+      <c r="F2007" t="inlineStr">
+        <is>
+          <t>6-32</t>
+        </is>
+      </c>
+      <c r="G2007" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2008" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2008" t="inlineStr">
+        <is>
+          <t>Garvaghey</t>
+        </is>
+      </c>
+      <c r="F2008" t="inlineStr">
+        <is>
+          <t>3-22</t>
+        </is>
+      </c>
+      <c r="G2008" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr">
+        <is>
+          <t>Lancashire</t>
+        </is>
+      </c>
+      <c r="D2009" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2009" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2009" t="inlineStr">
+        <is>
+          <t>2-28</t>
+        </is>
+      </c>
+      <c r="G2009" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2010" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2010" t="inlineStr">
+        <is>
+          <t>Enniscrone</t>
+        </is>
+      </c>
+      <c r="F2010" t="inlineStr">
+        <is>
+          <t>8-19</t>
+        </is>
+      </c>
+      <c r="G2010" t="inlineStr">
+        <is>
+          <t>0-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2011" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2011" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2011" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+      <c r="G2011" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Michael Cusack (Senior C) Cup</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>Colaiste Naomh Cormac</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr">
+        <is>
+          <t>St Patrick's High School Keady</t>
+        </is>
+      </c>
+      <c r="D2012" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2012" t="inlineStr">
+        <is>
+          <t>Gaeil Colmcille GFC (Grangegodden)</t>
+        </is>
+      </c>
+      <c r="F2012" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="G2012" t="inlineStr">
+        <is>
+          <t>3-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Michael Cusack (Senior C) Cup</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>St Josephs Borrisoleigh</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr">
+        <is>
+          <t>Garbally College Ballinasloe</t>
+        </is>
+      </c>
+      <c r="D2013" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2013" t="inlineStr">
+        <is>
+          <t>Banagher</t>
+        </is>
+      </c>
+      <c r="F2013" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+      <c r="G2013" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Niall McInerney (Senior D) Cup</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>St Michaels College Enniskillen</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
+        <is>
+          <t>Scoil Aireagal Ballyhale</t>
+        </is>
+      </c>
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2014" t="inlineStr">
+        <is>
+          <t>Abbottstown - GAA Centre of Excellence</t>
+        </is>
+      </c>
+      <c r="F2014" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+      <c r="G2014" t="inlineStr">
+        <is>
+          <t>3-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Paddy Buggy (Senior B) Cup</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>Portumna Community School</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr">
+        <is>
+          <t>Tralee CBS</t>
+        </is>
+      </c>
+      <c r="D2015" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2015" t="inlineStr">
+        <is>
+          <t>Tulla</t>
+        </is>
+      </c>
+      <c r="F2015" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="G2015" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Paddy Buggy (Senior B) Cup</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>Colaiste Eamann Ris Callan</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr">
+        <is>
+          <t>St Patricks Maghera</t>
+        </is>
+      </c>
+      <c r="D2016" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2016" t="inlineStr">
+        <is>
+          <t>Ml. Fay Park</t>
+        </is>
+      </c>
+      <c r="F2016" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+      <c r="G2016" t="inlineStr">
+        <is>
+          <t>2-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>Masita GAA Post Primary Schools Croke Cup (Senior A Hurling)</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>St. Kieran's College</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr">
+        <is>
+          <t>Nenagh C.B.S</t>
+        </is>
+      </c>
+      <c r="D2017" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2017" t="inlineStr">
+        <is>
+          <t>Rathdowney</t>
+        </is>
+      </c>
+      <c r="F2017" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+      <c r="G2017" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>Masita GAA Post Primary Schools Croke Cup (Senior A Hurling)</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>Presentation College Athenry</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr">
+        <is>
+          <t>St. Flannans College Ennis</t>
+        </is>
+      </c>
+      <c r="D2018" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="E2018" t="inlineStr">
+        <is>
+          <t>Kilbeacanty</t>
+        </is>
+      </c>
+      <c r="F2018" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2018" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-08
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2018"/>
+  <dimension ref="A1:G2025"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71474,6 +71474,265 @@
         </is>
       </c>
     </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1B</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2019" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E2019" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2019" t="inlineStr">
+        <is>
+          <t>0-26</t>
+        </is>
+      </c>
+      <c r="G2019" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1B</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2020" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E2020" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Newbridge</t>
+        </is>
+      </c>
+      <c r="F2020" t="inlineStr">
+        <is>
+          <t>3-22</t>
+        </is>
+      </c>
+      <c r="G2020" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2021" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E2021" t="inlineStr">
+        <is>
+          <t>Austin Stack Park</t>
+        </is>
+      </c>
+      <c r="F2021" t="inlineStr">
+        <is>
+          <t>6-24</t>
+        </is>
+      </c>
+      <c r="G2021" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2022" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E2022" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park</t>
+        </is>
+      </c>
+      <c r="F2022" t="inlineStr">
+        <is>
+          <t>0-28</t>
+        </is>
+      </c>
+      <c r="G2022" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="D2023" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E2023" t="inlineStr">
+        <is>
+          <t>TEG Cusack Park</t>
+        </is>
+      </c>
+      <c r="F2023" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+      <c r="G2023" t="inlineStr">
+        <is>
+          <t>3-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2024" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E2024" t="inlineStr">
+        <is>
+          <t>Letterkenny</t>
+        </is>
+      </c>
+      <c r="F2024" t="inlineStr">
+        <is>
+          <t>0-14</t>
+        </is>
+      </c>
+      <c r="G2024" t="inlineStr">
+        <is>
+          <t>0-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2025" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E2025" t="inlineStr">
+        <is>
+          <t>Brewster Park</t>
+        </is>
+      </c>
+      <c r="F2025" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+      <c r="G2025" t="inlineStr">
+        <is>
+          <t>5-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-14
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2025"/>
+  <dimension ref="A1:G2035"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -71733,6 +71733,376 @@
         </is>
       </c>
     </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2026" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2026" t="inlineStr">
+        <is>
+          <t>Austin Stack Park</t>
+        </is>
+      </c>
+      <c r="F2026" t="inlineStr">
+        <is>
+          <t>2-29</t>
+        </is>
+      </c>
+      <c r="G2026" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2027" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2027" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2027" t="inlineStr">
+        <is>
+          <t>1-25</t>
+        </is>
+      </c>
+      <c r="G2027" t="inlineStr">
+        <is>
+          <t>2-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="D2028" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2028" t="inlineStr">
+        <is>
+          <t>DEFY Pairc Mhuire, Ardee</t>
+        </is>
+      </c>
+      <c r="F2028" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="G2028" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="D2029" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2029" t="inlineStr">
+        <is>
+          <t>Páirc Uí Rinn</t>
+        </is>
+      </c>
+      <c r="F2029" t="inlineStr">
+        <is>
+          <t>1-31</t>
+        </is>
+      </c>
+      <c r="G2029" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2030" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2030" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2030" t="inlineStr">
+        <is>
+          <t>3-24</t>
+        </is>
+      </c>
+      <c r="G2030" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2031" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2031" t="inlineStr">
+        <is>
+          <t>Brewster Park</t>
+        </is>
+      </c>
+      <c r="F2031" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+      <c r="G2031" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D2032" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2032" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park</t>
+        </is>
+      </c>
+      <c r="F2032" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+      <c r="G2032" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland PPS Br Edmund Ignatius Rice Cup (Senior D Football)</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>Largy College Clones</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>Rice College Ennis</t>
+        </is>
+      </c>
+      <c r="D2033" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2033" t="inlineStr">
+        <is>
+          <t>Connacht GAA Centre</t>
+        </is>
+      </c>
+      <c r="F2033" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+      <c r="G2033" t="inlineStr">
+        <is>
+          <t>0-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland PPS Dr Eamonn O'Sullivan Cup (Senior C Football)</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>Balla Secondary School</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>St Ciaran's, Ballygawley</t>
+        </is>
+      </c>
+      <c r="D2034" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2034" t="inlineStr">
+        <is>
+          <t>Father Tierney Park, Ballyshannon</t>
+        </is>
+      </c>
+      <c r="F2034" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="G2034" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland PPS Paddy Drummond Cup (Senior B Football)</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>St. Nathy's College Ballaghaderreen</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>Cnoc Mhuire Granard</t>
+        </is>
+      </c>
+      <c r="D2035" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E2035" t="inlineStr">
+        <is>
+          <t>Páirc Sheáin Uí Eislin, Ballinamore</t>
+        </is>
+      </c>
+      <c r="F2035" t="inlineStr">
+        <is>
+          <t>1-9</t>
+        </is>
+      </c>
+      <c r="G2035" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-15
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2035"/>
+  <dimension ref="A1:G2045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72103,6 +72103,376 @@
         </is>
       </c>
     </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2036" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2036" t="inlineStr">
+        <is>
+          <t>King &amp; Moffatt Dr. Hyde Park</t>
+        </is>
+      </c>
+      <c r="F2036" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2036" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2037" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2037" t="inlineStr">
+        <is>
+          <t>Páirc Grattan, Inniskeen</t>
+        </is>
+      </c>
+      <c r="F2037" t="inlineStr">
+        <is>
+          <t>2-9</t>
+        </is>
+      </c>
+      <c r="G2037" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2038" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2038" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park</t>
+        </is>
+      </c>
+      <c r="F2038" t="inlineStr">
+        <is>
+          <t>3-15</t>
+        </is>
+      </c>
+      <c r="G2038" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2039" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2039" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2039" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+      <c r="G2039" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2040" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2040" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2040" t="inlineStr">
+        <is>
+          <t>0-21</t>
+        </is>
+      </c>
+      <c r="G2040" t="inlineStr">
+        <is>
+          <t>2-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2041" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2041" t="inlineStr">
+        <is>
+          <t>TEG Cusack Park</t>
+        </is>
+      </c>
+      <c r="F2041" t="inlineStr">
+        <is>
+          <t>4-21</t>
+        </is>
+      </c>
+      <c r="G2041" t="inlineStr">
+        <is>
+          <t>3-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="D2042" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2042" t="inlineStr">
+        <is>
+          <t>Cappoquin Logistics Fraher Field, Dungarvan</t>
+        </is>
+      </c>
+      <c r="F2042" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+      <c r="G2042" t="inlineStr">
+        <is>
+          <t>4-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2043" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2043" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2043" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+      <c r="G2043" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2044" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2044" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2044" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+      <c r="G2044" t="inlineStr">
+        <is>
+          <t>0-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1A</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2045" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2045" t="inlineStr">
+        <is>
+          <t>Azzurri Walsh Park, Waterford</t>
+        </is>
+      </c>
+      <c r="F2045" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G2045" t="inlineStr">
+        <is>
+          <t>2-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-17
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2045"/>
+  <dimension ref="A1:G2047"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72473,6 +72473,80 @@
         </is>
       </c>
     </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland PPS Hogan Cup (Senior A Football)</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>Colaiste Mhuire Mullingar</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>Tralee CBS</t>
+        </is>
+      </c>
+      <c r="D2046" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="E2046" t="inlineStr">
+        <is>
+          <t>Croke Park</t>
+        </is>
+      </c>
+      <c r="F2046" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+      <c r="G2046" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>Masita GAA Post Primary Schools Croke Cup (Senior A Hurling)</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>Presentation College Athenry</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>St. Kieran's College</t>
+        </is>
+      </c>
+      <c r="D2047" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="E2047" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2047" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+      <c r="G2047" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-20
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2047"/>
+  <dimension ref="A1:G2049"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72547,6 +72547,80 @@
         </is>
       </c>
     </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2048" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E2048" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2048" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+      <c r="G2048" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Michael Cusack (Senior C) Cup</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>Colaiste Naomh Cormac</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>St Josephs Borrisoleigh</t>
+        </is>
+      </c>
+      <c r="D2049" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E2049" t="inlineStr">
+        <is>
+          <t>Borrisokane</t>
+        </is>
+      </c>
+      <c r="F2049" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="G2049" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-21
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2049"/>
+  <dimension ref="A1:G2066"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72621,6 +72621,635 @@
         </is>
       </c>
     </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1A</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="D2050" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2050" t="inlineStr">
+        <is>
+          <t>SuperValu Páirc Uí Chaoimh</t>
+        </is>
+      </c>
+      <c r="F2050" t="inlineStr">
+        <is>
+          <t>6-26</t>
+        </is>
+      </c>
+      <c r="G2050" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1A</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2051" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2051" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2051" t="inlineStr">
+        <is>
+          <t>2-27</t>
+        </is>
+      </c>
+      <c r="G2051" t="inlineStr">
+        <is>
+          <t>0-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1A</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="D2052" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2052" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2052" t="inlineStr">
+        <is>
+          <t>2-27</t>
+        </is>
+      </c>
+      <c r="G2052" t="inlineStr">
+        <is>
+          <t>3-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1B</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2053" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2053" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park</t>
+        </is>
+      </c>
+      <c r="F2053" t="inlineStr">
+        <is>
+          <t>2-14</t>
+        </is>
+      </c>
+      <c r="G2053" t="inlineStr">
+        <is>
+          <t>0-34</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1B</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="D2054" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2054" t="inlineStr">
+        <is>
+          <t>Páirc Esler, Newry</t>
+        </is>
+      </c>
+      <c r="F2054" t="inlineStr">
+        <is>
+          <t>3-22</t>
+        </is>
+      </c>
+      <c r="G2054" t="inlineStr">
+        <is>
+          <t>3-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1B</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="D2055" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2055" t="inlineStr">
+        <is>
+          <t>Chadwicks Wexford Park</t>
+        </is>
+      </c>
+      <c r="F2055" t="inlineStr">
+        <is>
+          <t>3-29</t>
+        </is>
+      </c>
+      <c r="G2055" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2056" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2056" t="inlineStr">
+        <is>
+          <t>McGovern Park, Ruislip</t>
+        </is>
+      </c>
+      <c r="F2056" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+      <c r="G2056" t="inlineStr">
+        <is>
+          <t>3-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2057" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2057" t="inlineStr">
+        <is>
+          <t>Hastings Insurance MacHale Park, Castlebar</t>
+        </is>
+      </c>
+      <c r="F2057" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+      <c r="G2057" t="inlineStr">
+        <is>
+          <t>2-37</t>
+        </is>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2058" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2058" t="inlineStr">
+        <is>
+          <t>Trim</t>
+        </is>
+      </c>
+      <c r="F2058" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+      <c r="G2058" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2059" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2059" t="inlineStr">
+        <is>
+          <t>BOX-IT Athletic Grounds, Armagh</t>
+        </is>
+      </c>
+      <c r="F2059" t="inlineStr">
+        <is>
+          <t>0-21</t>
+        </is>
+      </c>
+      <c r="G2059" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2060" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2060" t="inlineStr">
+        <is>
+          <t>King &amp; Moffatt Dr. Hyde Park</t>
+        </is>
+      </c>
+      <c r="F2060" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+      <c r="G2060" t="inlineStr">
+        <is>
+          <t>3-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2061" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2061" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2061" t="inlineStr">
+        <is>
+          <t>3-27</t>
+        </is>
+      </c>
+      <c r="G2061" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="D2062" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2062" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2062" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+      <c r="G2062" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>Lancashire</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="D2063" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2063" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2063" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="G2063" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="D2064" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2064" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2064" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+      <c r="G2064" t="inlineStr">
+        <is>
+          <t>4-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Niall McInerney (Senior D) Cup</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>Mount Sion CBS Post Primary</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr">
+        <is>
+          <t>Scoil Aireagal Ballyhale</t>
+        </is>
+      </c>
+      <c r="D2065" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2065" t="inlineStr">
+        <is>
+          <t>O Kennedy Park, New Ross</t>
+        </is>
+      </c>
+      <c r="F2065" t="inlineStr">
+        <is>
+          <t>3-18</t>
+        </is>
+      </c>
+      <c r="G2065" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>Masita All-Ireland Post Primary Schools Paddy Buggy (Senior B) Cup</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>St Patricks Maghera</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr">
+        <is>
+          <t>Tralee CBS</t>
+        </is>
+      </c>
+      <c r="D2066" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E2066" t="inlineStr">
+        <is>
+          <t>Kinnegad</t>
+        </is>
+      </c>
+      <c r="F2066" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+      <c r="G2066" t="inlineStr">
+        <is>
+          <t>2-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-22
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2066"/>
+  <dimension ref="A1:G2082"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73250,6 +73250,598 @@
         </is>
       </c>
     </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2067" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2067" t="inlineStr">
+        <is>
+          <t>BOX-IT Athletic Grounds, Armagh</t>
+        </is>
+      </c>
+      <c r="F2067" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+      <c r="G2067" t="inlineStr">
+        <is>
+          <t>0-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2068" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2068" t="inlineStr">
+        <is>
+          <t>Pearse Stadium</t>
+        </is>
+      </c>
+      <c r="F2068" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="G2068" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2069" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2069" t="inlineStr">
+        <is>
+          <t>Hastings Insurance MacHale Park, Castlebar</t>
+        </is>
+      </c>
+      <c r="F2069" t="inlineStr">
+        <is>
+          <t>4-26</t>
+        </is>
+      </c>
+      <c r="G2069" t="inlineStr">
+        <is>
+          <t>2-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2070" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2070" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2070" t="inlineStr">
+        <is>
+          <t>3-16</t>
+        </is>
+      </c>
+      <c r="G2070" t="inlineStr">
+        <is>
+          <t>3-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2071" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2071" t="inlineStr">
+        <is>
+          <t>Find Insurance Celtic Park, Derry</t>
+        </is>
+      </c>
+      <c r="F2071" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+      <c r="G2071" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2072" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2072" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Newbridge</t>
+        </is>
+      </c>
+      <c r="F2072" t="inlineStr">
+        <is>
+          <t>0-25</t>
+        </is>
+      </c>
+      <c r="G2072" t="inlineStr">
+        <is>
+          <t>1-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2073" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2073" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park</t>
+        </is>
+      </c>
+      <c r="F2073" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+      <c r="G2073" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2074" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2074" t="inlineStr">
+        <is>
+          <t>O'Neills Healy Park, Omagh</t>
+        </is>
+      </c>
+      <c r="F2074" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+      <c r="G2074" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2075" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2075" t="inlineStr">
+        <is>
+          <t>Páirc Esler, Newry</t>
+        </is>
+      </c>
+      <c r="F2075" t="inlineStr">
+        <is>
+          <t>0-24</t>
+        </is>
+      </c>
+      <c r="G2075" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2076" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2076" t="inlineStr">
+        <is>
+          <t>Mick Neville Park Rathkeale</t>
+        </is>
+      </c>
+      <c r="F2076" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+      <c r="G2076" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="D2077" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2077" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2077" t="inlineStr">
+        <is>
+          <t>2-23</t>
+        </is>
+      </c>
+      <c r="G2077" t="inlineStr">
+        <is>
+          <t>0-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2078" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2078" t="inlineStr">
+        <is>
+          <t>Chadwicks Wexford Park</t>
+        </is>
+      </c>
+      <c r="F2078" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+      <c r="G2078" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D2079" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2079" t="inlineStr">
+        <is>
+          <t>Erins Own, Cargin (Toomebridge)</t>
+        </is>
+      </c>
+      <c r="F2079" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+      <c r="G2079" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="D2080" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2080" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park</t>
+        </is>
+      </c>
+      <c r="F2080" t="inlineStr">
+        <is>
+          <t>4-22</t>
+        </is>
+      </c>
+      <c r="G2080" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2081" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2081" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2081" t="inlineStr">
+        <is>
+          <t>2-21</t>
+        </is>
+      </c>
+      <c r="G2081" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="D2082" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E2082" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2082" t="inlineStr">
+        <is>
+          <t>4-19</t>
+        </is>
+      </c>
+      <c r="G2082" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-28
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2082"/>
+  <dimension ref="A1:G2087"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73842,6 +73842,191 @@
         </is>
       </c>
     </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2083" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="E2083" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2083" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+      <c r="G2083" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2084" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="E2084" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park</t>
+        </is>
+      </c>
+      <c r="F2084" t="inlineStr">
+        <is>
+          <t>3-18</t>
+        </is>
+      </c>
+      <c r="G2084" t="inlineStr">
+        <is>
+          <t>0-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2085" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="E2085" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2085" t="inlineStr">
+        <is>
+          <t>3-16</t>
+        </is>
+      </c>
+      <c r="G2085" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 4</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2086" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="E2086" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2086" t="inlineStr">
+        <is>
+          <t>2-21</t>
+        </is>
+      </c>
+      <c r="G2086" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>Fulfil GAA Hurling All-Ireland U20C Championship - Andrew O'Neill Cup</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2087" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="E2087" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2087" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+      <c r="G2087" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-29
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2087"/>
+  <dimension ref="A1:G2094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74027,6 +74027,265 @@
         </is>
       </c>
     </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 3</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2088" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="E2088" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2088" t="inlineStr">
+        <is>
+          <t>0-21</t>
+        </is>
+      </c>
+      <c r="G2088" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2089" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="E2089" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2089" t="inlineStr">
+        <is>
+          <t>3-20</t>
+        </is>
+      </c>
+      <c r="G2089" t="inlineStr">
+        <is>
+          <t>2-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 2</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2090" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="E2090" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2090" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+      <c r="G2090" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>Fulfil  GAA Hurling All-Ireland U20B Championship - Richie McElligott Cup</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2091" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="E2091" t="inlineStr">
+        <is>
+          <t>Abbottstown - GAA Centre of Excellence</t>
+        </is>
+      </c>
+      <c r="F2091" t="inlineStr">
+        <is>
+          <t>5-11</t>
+        </is>
+      </c>
+      <c r="G2091" t="inlineStr">
+        <is>
+          <t>4-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>Fulfil  GAA Hurling All-Ireland U20B Championship - Richie McElligott Cup</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2092" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="E2092" t="inlineStr">
+        <is>
+          <t>King &amp; Moffatt Dr. Hyde Park</t>
+        </is>
+      </c>
+      <c r="F2092" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2092" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>Fulfil GAA Hurling All-Ireland U20C Championship - Andrew O'Neill Cup</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2093" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="E2093" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2093" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+      <c r="G2093" t="inlineStr">
+        <is>
+          <t>3-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr">
+        <is>
+          <t>Fulfil GAA Hurling All-Ireland U20C Championship - Andrew O'Neill Cup</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2094" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="E2094" t="inlineStr">
+        <is>
+          <t>Connacht Centre of Excellence</t>
+        </is>
+      </c>
+      <c r="F2094" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="G2094" t="inlineStr">
+        <is>
+          <t>6-5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-03-30
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2094"/>
+  <dimension ref="A1:G2095"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74286,6 +74286,43 @@
         </is>
       </c>
     </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>Allianz Football League Roinn 1</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2095" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
+      <c r="E2095" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2095" t="inlineStr">
+        <is>
+          <t>2-10</t>
+        </is>
+      </c>
+      <c r="G2095" t="inlineStr">
+        <is>
+          <t>3-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-04
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2095"/>
+  <dimension ref="A1:G2098"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74323,6 +74323,117 @@
         </is>
       </c>
     </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr">
+        <is>
+          <t>Fulfil  GAA Hurling All-Ireland U20B Championship - Richie McElligott Cup</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2096" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="E2096" t="inlineStr">
+        <is>
+          <t>Find Insurance Owenbeg</t>
+        </is>
+      </c>
+      <c r="F2096" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="G2096" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>Fulfil  GAA Hurling All-Ireland U20B Championship - Richie McElligott Cup</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2097" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="E2097" t="inlineStr">
+        <is>
+          <t>Garvaghey</t>
+        </is>
+      </c>
+      <c r="F2097" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2097" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr">
+        <is>
+          <t>Fulfil GAA Hurling All-Ireland U20C Championship - Andrew O'Neill Cup</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2098" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="E2098" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2098" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="G2098" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-05
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2098"/>
+  <dimension ref="A1:G2101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74434,6 +74434,117 @@
         </is>
       </c>
     </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1A</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2099" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="E2099" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2099" t="inlineStr">
+        <is>
+          <t>1-27</t>
+        </is>
+      </c>
+      <c r="G2099" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr">
+        <is>
+          <t>Allianz Hurling League Roinn 1B</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2100" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="E2100" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2100" t="inlineStr">
+        <is>
+          <t>2-26</t>
+        </is>
+      </c>
+      <c r="G2100" t="inlineStr">
+        <is>
+          <t>3-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>Fulfil GAA Hurling All-Ireland U20C Championship - Andrew O'Neill Cup</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2101" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="E2101" t="inlineStr">
+        <is>
+          <t>VBC Cloghan, Castleblayney</t>
+        </is>
+      </c>
+      <c r="F2101" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+      <c r="G2101" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-11
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2101"/>
+  <dimension ref="A1:G2108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74545,6 +74545,265 @@
         </is>
       </c>
     </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr">
+        <is>
+          <t>Connacht GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2102" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2102" t="inlineStr">
+        <is>
+          <t>McGovern Park, Ruislip</t>
+        </is>
+      </c>
+      <c r="F2102" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2102" t="inlineStr">
+        <is>
+          <t>0-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="D2103" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2103" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2103" t="inlineStr">
+        <is>
+          <t>3-14</t>
+        </is>
+      </c>
+      <c r="G2103" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr">
+        <is>
+          <t>Lancashire</t>
+        </is>
+      </c>
+      <c r="D2104" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2104" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2104" t="inlineStr">
+        <is>
+          <t>5-21</t>
+        </is>
+      </c>
+      <c r="G2104" t="inlineStr">
+        <is>
+          <t>1-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="D2105" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2105" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2105" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+      <c r="G2105" t="inlineStr">
+        <is>
+          <t>2-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2106" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2106" t="inlineStr">
+        <is>
+          <t>BOX-IT Athletic Grounds, Armagh</t>
+        </is>
+      </c>
+      <c r="F2106" t="inlineStr">
+        <is>
+          <t>2-7</t>
+        </is>
+      </c>
+      <c r="G2106" t="inlineStr">
+        <is>
+          <t>2-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2107" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2107" t="inlineStr">
+        <is>
+          <t>Dowdallshill, Dundalk</t>
+        </is>
+      </c>
+      <c r="F2107" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+      <c r="G2107" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="D2108" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2108" t="inlineStr">
+        <is>
+          <t>Garvaghey</t>
+        </is>
+      </c>
+      <c r="F2108" t="inlineStr">
+        <is>
+          <t>4-10</t>
+        </is>
+      </c>
+      <c r="G2108" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-12
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2108"/>
+  <dimension ref="A1:G2119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74804,6 +74804,413 @@
         </is>
       </c>
     </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2109" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="E2109" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park</t>
+        </is>
+      </c>
+      <c r="F2109" t="inlineStr">
+        <is>
+          <t>0-12</t>
+        </is>
+      </c>
+      <c r="G2109" t="inlineStr">
+        <is>
+          <t>3-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2110" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2110" t="inlineStr">
+        <is>
+          <t>O'Donnell Park, Letterkenny</t>
+        </is>
+      </c>
+      <c r="F2110" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+      <c r="G2110" t="inlineStr">
+        <is>
+          <t>1-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2111" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2111" t="inlineStr">
+        <is>
+          <t>Trim</t>
+        </is>
+      </c>
+      <c r="F2111" t="inlineStr">
+        <is>
+          <t>0-12</t>
+        </is>
+      </c>
+      <c r="G2111" t="inlineStr">
+        <is>
+          <t>3-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2112" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2112" t="inlineStr">
+        <is>
+          <t>Find Insurance Celtic Park, Derry</t>
+        </is>
+      </c>
+      <c r="F2112" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+      <c r="G2112" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>Connacht GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="D2113" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2113" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2113" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+      <c r="G2113" t="inlineStr">
+        <is>
+          <t>3-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr">
+        <is>
+          <t>Connacht GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2114" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2114" t="inlineStr">
+        <is>
+          <t>Gaelic Park, New York</t>
+        </is>
+      </c>
+      <c r="F2114" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+      <c r="G2114" t="inlineStr">
+        <is>
+          <t>5-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2115" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2115" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park</t>
+        </is>
+      </c>
+      <c r="F2115" t="inlineStr">
+        <is>
+          <t>1-7</t>
+        </is>
+      </c>
+      <c r="G2115" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2116" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2116" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2116" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+      <c r="G2116" t="inlineStr">
+        <is>
+          <t>5-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>Munster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2117" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2117" t="inlineStr">
+        <is>
+          <t>SuperValu Páirc Uí Chaoimh</t>
+        </is>
+      </c>
+      <c r="F2117" t="inlineStr">
+        <is>
+          <t>4-16</t>
+        </is>
+      </c>
+      <c r="G2117" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr">
+        <is>
+          <t>Munster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2118" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2118" t="inlineStr">
+        <is>
+          <t>Cappoquin Logistics Fraher Field</t>
+        </is>
+      </c>
+      <c r="F2118" t="inlineStr">
+        <is>
+          <t>1-7</t>
+        </is>
+      </c>
+      <c r="G2118" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2119" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="E2119" t="inlineStr">
+        <is>
+          <t>BOX-IT Athletic Grounds, Armagh</t>
+        </is>
+      </c>
+      <c r="F2119" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+      <c r="G2119" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-18
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2119"/>
+  <dimension ref="A1:G2128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75211,6 +75211,339 @@
         </is>
       </c>
     </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2120" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2120" t="inlineStr">
+        <is>
+          <t>Ballyforan</t>
+        </is>
+      </c>
+      <c r="F2120" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="G2120" t="inlineStr">
+        <is>
+          <t>0-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2121" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2121" t="inlineStr">
+        <is>
+          <t>Dunloy</t>
+        </is>
+      </c>
+      <c r="F2121" t="inlineStr">
+        <is>
+          <t>0-23</t>
+        </is>
+      </c>
+      <c r="G2121" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2122" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2122" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park</t>
+        </is>
+      </c>
+      <c r="F2122" t="inlineStr">
+        <is>
+          <t>4-17</t>
+        </is>
+      </c>
+      <c r="G2122" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="D2123" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2123" t="inlineStr">
+        <is>
+          <t>Pearse Stadium</t>
+        </is>
+      </c>
+      <c r="F2123" t="inlineStr">
+        <is>
+          <t>3-25</t>
+        </is>
+      </c>
+      <c r="G2123" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2124" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2124" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Newbridge</t>
+        </is>
+      </c>
+      <c r="F2124" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+      <c r="G2124" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2125" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2125" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park</t>
+        </is>
+      </c>
+      <c r="F2125" t="inlineStr">
+        <is>
+          <t>4-22</t>
+        </is>
+      </c>
+      <c r="G2125" t="inlineStr">
+        <is>
+          <t>2-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2126" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2126" t="inlineStr">
+        <is>
+          <t>Patrick McManus Park, Kinawley</t>
+        </is>
+      </c>
+      <c r="F2126" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2126" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2127" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2127" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2127" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2127" t="inlineStr">
+        <is>
+          <t>1-31</t>
+        </is>
+      </c>
+      <c r="G2127" t="inlineStr">
+        <is>
+          <t>0-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2128" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2128" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="D2128" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2128" t="inlineStr">
+        <is>
+          <t>Find Insurance Celtic Park, Derry</t>
+        </is>
+      </c>
+      <c r="F2128" t="inlineStr">
+        <is>
+          <t>2-23</t>
+        </is>
+      </c>
+      <c r="G2128" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-19
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2128"/>
+  <dimension ref="A1:G2142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75544,6 +75544,524 @@
         </is>
       </c>
     </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2129" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="D2129" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2129" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2129" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="G2129" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2130" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2130" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2130" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2130" t="inlineStr">
+        <is>
+          <t>Austin Stack Park</t>
+        </is>
+      </c>
+      <c r="F2130" t="inlineStr">
+        <is>
+          <t>5-18</t>
+        </is>
+      </c>
+      <c r="G2130" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2131" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2131" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2131" t="inlineStr">
+        <is>
+          <t>McGovern Park, Ruislip</t>
+        </is>
+      </c>
+      <c r="F2131" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+      <c r="G2131" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2132">
+      <c r="A2132" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2132" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="C2132" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2132" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2132" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park</t>
+        </is>
+      </c>
+      <c r="F2132" t="inlineStr">
+        <is>
+          <t>0-25</t>
+        </is>
+      </c>
+      <c r="G2132" t="inlineStr">
+        <is>
+          <t>4-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2133" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2133" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2133" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park</t>
+        </is>
+      </c>
+      <c r="F2133" t="inlineStr">
+        <is>
+          <t>1-25</t>
+        </is>
+      </c>
+      <c r="G2133" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2134">
+      <c r="A2134" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2134" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2134" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2134" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2134" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2134" t="inlineStr">
+        <is>
+          <t>2-14</t>
+        </is>
+      </c>
+      <c r="G2134" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2135" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2135" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2135" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Park</t>
+        </is>
+      </c>
+      <c r="F2135" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2135" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2136" t="inlineStr">
+        <is>
+          <t>Lancashire</t>
+        </is>
+      </c>
+      <c r="C2136" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="D2136" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2136" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2136" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+      <c r="G2136" t="inlineStr">
+        <is>
+          <t>2-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2137" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2137" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2137" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2137" t="inlineStr">
+        <is>
+          <t>3-22</t>
+        </is>
+      </c>
+      <c r="G2137" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2138" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="C2138" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2138" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2138" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2138" t="inlineStr">
+        <is>
+          <t>3-12</t>
+        </is>
+      </c>
+      <c r="G2138" t="inlineStr">
+        <is>
+          <t>4-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2139" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="D2139" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2139" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2139" t="inlineStr">
+        <is>
+          <t>2-33</t>
+        </is>
+      </c>
+      <c r="G2139" t="inlineStr">
+        <is>
+          <t>4-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="C2140" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2140" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2140" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2140" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+      <c r="G2140" t="inlineStr">
+        <is>
+          <t>0-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C2141" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2141" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2141" t="inlineStr">
+        <is>
+          <t>Hastings Insurance MacHale Park, Castlebar</t>
+        </is>
+      </c>
+      <c r="F2141" t="inlineStr">
+        <is>
+          <t>1-25</t>
+        </is>
+      </c>
+      <c r="G2141" t="inlineStr">
+        <is>
+          <t>5-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2142" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2142" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="E2142" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2142" t="inlineStr">
+        <is>
+          <t>0-27</t>
+        </is>
+      </c>
+      <c r="G2142" t="inlineStr">
+        <is>
+          <t>2-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-24
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2142"/>
+  <dimension ref="A1:G2143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76062,6 +76062,43 @@
         </is>
       </c>
     </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2143" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D2143" t="inlineStr">
+        <is>
+          <t>24/04/2026</t>
+        </is>
+      </c>
+      <c r="E2143" t="inlineStr">
+        <is>
+          <t>Connacht GAA Centre</t>
+        </is>
+      </c>
+      <c r="F2143" t="inlineStr">
+        <is>
+          <t>1-8</t>
+        </is>
+      </c>
+      <c r="G2143" t="inlineStr">
+        <is>
+          <t>4-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-25
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2143"/>
+  <dimension ref="A1:G2154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76099,6 +76099,413 @@
         </is>
       </c>
     </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2144" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2144" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2144" t="inlineStr">
+        <is>
+          <t>Find Insurance Celtic Park, Derry</t>
+        </is>
+      </c>
+      <c r="F2144" t="inlineStr">
+        <is>
+          <t>2-23</t>
+        </is>
+      </c>
+      <c r="G2144" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2145" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2145" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2145" t="inlineStr">
+        <is>
+          <t>Ballyforan</t>
+        </is>
+      </c>
+      <c r="F2145" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2145" t="inlineStr">
+        <is>
+          <t>4-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr">
+        <is>
+          <t>Connacht GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2146" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2146" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2146" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2146" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="G2146" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2147" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D2147" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2147" t="inlineStr">
+        <is>
+          <t>Páirc Esler, Newry</t>
+        </is>
+      </c>
+      <c r="F2147" t="inlineStr">
+        <is>
+          <t>2-23</t>
+        </is>
+      </c>
+      <c r="G2147" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2148" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="D2148" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2148" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park</t>
+        </is>
+      </c>
+      <c r="F2148" t="inlineStr">
+        <is>
+          <t>2-23</t>
+        </is>
+      </c>
+      <c r="G2148" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="C2149" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2149" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2149" t="inlineStr">
+        <is>
+          <t>TEG Cusack Park</t>
+        </is>
+      </c>
+      <c r="F2149" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G2149" t="inlineStr">
+        <is>
+          <t>4-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2150" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="C2150" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2150" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2150" t="inlineStr">
+        <is>
+          <t>UPMC Nowlan Park</t>
+        </is>
+      </c>
+      <c r="F2150" t="inlineStr">
+        <is>
+          <t>5-21</t>
+        </is>
+      </c>
+      <c r="G2150" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr">
+        <is>
+          <t>Munster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2151" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2151" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2151" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2151" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+      <c r="G2151" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="inlineStr">
+        <is>
+          <t>Munster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2152" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="C2152" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2152" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2152" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2152" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+      <c r="G2152" t="inlineStr">
+        <is>
+          <t>4-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2153" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2153" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2153" t="inlineStr">
+        <is>
+          <t>Dowdallshill, Dundalk</t>
+        </is>
+      </c>
+      <c r="F2153" t="inlineStr">
+        <is>
+          <t>2-14</t>
+        </is>
+      </c>
+      <c r="G2153" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2154" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2154" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2154" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2154" t="inlineStr">
+        <is>
+          <t>Brewster Park</t>
+        </is>
+      </c>
+      <c r="F2154" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+      <c r="G2154" t="inlineStr">
+        <is>
+          <t>2-32</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-26
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2154"/>
+  <dimension ref="A1:G2166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76506,6 +76506,450 @@
         </is>
       </c>
     </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2155" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2155" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2155" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2155" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="G2155" t="inlineStr">
+        <is>
+          <t>2-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="inlineStr">
+        <is>
+          <t>Connacht GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2156" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C2156" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2156" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2156" t="inlineStr">
+        <is>
+          <t>Hastings Insurance MacHale Park, Castlebar</t>
+        </is>
+      </c>
+      <c r="F2156" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2156" t="inlineStr">
+        <is>
+          <t>2-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2157" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D2157" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2157" t="inlineStr">
+        <is>
+          <t>Connacht GAA Centre</t>
+        </is>
+      </c>
+      <c r="F2157" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2157" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2158" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2158" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="D2158" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2158" t="inlineStr">
+        <is>
+          <t>Parnell Park</t>
+        </is>
+      </c>
+      <c r="F2158" t="inlineStr">
+        <is>
+          <t>3-24</t>
+        </is>
+      </c>
+      <c r="G2158" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2159" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="D2159" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2159" t="inlineStr">
+        <is>
+          <t>Pearse Stadium</t>
+        </is>
+      </c>
+      <c r="F2159" t="inlineStr">
+        <is>
+          <t>2-26</t>
+        </is>
+      </c>
+      <c r="G2159" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2160" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2160" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2160" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2160" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2160" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="G2160" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="C2161" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="D2161" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2161" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2161" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+      <c r="G2161" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2162" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2162" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2162" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2162" t="inlineStr">
+        <is>
+          <t>SuperValu Páirc Uí Chaoimh</t>
+        </is>
+      </c>
+      <c r="F2162" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+      <c r="G2162" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2163" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2163" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2163" t="inlineStr">
+        <is>
+          <t>Azzurri Walsh Park, Waterford</t>
+        </is>
+      </c>
+      <c r="F2163" t="inlineStr">
+        <is>
+          <t>3-24</t>
+        </is>
+      </c>
+      <c r="G2163" t="inlineStr">
+        <is>
+          <t>1-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2164" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2164" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2164" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2164" t="inlineStr">
+        <is>
+          <t>Brewster Park, Enniskillen</t>
+        </is>
+      </c>
+      <c r="F2164" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+      <c r="G2164" t="inlineStr">
+        <is>
+          <t>2-34</t>
+        </is>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2165" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2165" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2165" t="inlineStr">
+        <is>
+          <t>Tubbercurry</t>
+        </is>
+      </c>
+      <c r="F2165" t="inlineStr">
+        <is>
+          <t>3-28</t>
+        </is>
+      </c>
+      <c r="G2165" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2166" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="C2166" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2166" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2166" t="inlineStr">
+        <is>
+          <t>O'Donnell Park, Letterkenny</t>
+        </is>
+      </c>
+      <c r="F2166" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+      <c r="G2166" t="inlineStr">
+        <is>
+          <t>3-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-27
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2166"/>
+  <dimension ref="A1:G2168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -76950,6 +76950,80 @@
         </is>
       </c>
     </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D2167" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2167" t="inlineStr">
+        <is>
+          <t>Connacht GAA Centre</t>
+        </is>
+      </c>
+      <c r="F2167" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2167" t="inlineStr">
+        <is>
+          <t>4-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr">
+        <is>
+          <t>Lancashire</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2168" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="E2168" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2168" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+      <c r="G2168" t="inlineStr">
+        <is>
+          <t>3-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-04-30
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2168"/>
+  <dimension ref="A1:G2171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77024,6 +77024,117 @@
         </is>
       </c>
     </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2169" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="E2169" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park, Carlow</t>
+        </is>
+      </c>
+      <c r="F2169" t="inlineStr">
+        <is>
+          <t>4-17</t>
+        </is>
+      </c>
+      <c r="G2169" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2170" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2170" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="D2170" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2170" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park, Portlaoise</t>
+        </is>
+      </c>
+      <c r="F2170" t="inlineStr">
+        <is>
+          <t>2-23</t>
+        </is>
+      </c>
+      <c r="G2170" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="C2171" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2171" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="E2171" t="inlineStr">
+        <is>
+          <t>TEG Cusack Park, Westmeath</t>
+        </is>
+      </c>
+      <c r="F2171" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G2171" t="inlineStr">
+        <is>
+          <t>4-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-02
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2171"/>
+  <dimension ref="A1:G2175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77135,6 +77135,154 @@
         </is>
       </c>
     </row>
+    <row r="2172">
+      <c r="A2172" t="inlineStr">
+        <is>
+          <t>Fulfil  GAA Hurling All-Ireland U20B Championship - Richie McElligott Cup</t>
+        </is>
+      </c>
+      <c r="B2172" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2172" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2172" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="E2172" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2172" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+      <c r="G2172" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr">
+        <is>
+          <t>Fulfil GAA Hurling All-Ireland U20C Championship - Andrew O'Neill Cup</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2173" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2173" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="E2173" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2173" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+      <c r="G2173" t="inlineStr">
+        <is>
+          <t>0-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2174" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2174" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2174" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="E2174" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park, Portlaoise</t>
+        </is>
+      </c>
+      <c r="F2174" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="G2174" t="inlineStr">
+        <is>
+          <t>0-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2175" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="D2175" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="E2175" t="inlineStr">
+        <is>
+          <t>BOX-IT Athletic Grounds, Armagh</t>
+        </is>
+      </c>
+      <c r="F2175" t="inlineStr">
+        <is>
+          <t>3-23</t>
+        </is>
+      </c>
+      <c r="G2175" t="inlineStr">
+        <is>
+          <t>1-30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-03
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2175"/>
+  <dimension ref="A1:G2178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77283,6 +77283,117 @@
         </is>
       </c>
     </row>
+    <row r="2176">
+      <c r="A2176" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2176" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2176" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2176" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="E2176" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park, Tullamore</t>
+        </is>
+      </c>
+      <c r="F2176" t="inlineStr">
+        <is>
+          <t>0-23</t>
+        </is>
+      </c>
+      <c r="G2176" t="inlineStr">
+        <is>
+          <t>2-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2177" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2177" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="E2177" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2177" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2177" t="inlineStr">
+        <is>
+          <t>2-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2178" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2178" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2178" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="E2178" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2178" t="inlineStr">
+        <is>
+          <t>3-33</t>
+        </is>
+      </c>
+      <c r="G2178" t="inlineStr">
+        <is>
+          <t>0-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-09
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2178"/>
+  <dimension ref="A1:G2198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -77394,6 +77394,746 @@
         </is>
       </c>
     </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2179" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2179" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2179" t="inlineStr">
+        <is>
+          <t>Austin Stack Park, Tralee</t>
+        </is>
+      </c>
+      <c r="F2179" t="inlineStr">
+        <is>
+          <t>8-25</t>
+        </is>
+      </c>
+      <c r="G2179" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2180" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="C2180" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="D2180" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2180" t="inlineStr">
+        <is>
+          <t>St Loman's Park, Trim</t>
+        </is>
+      </c>
+      <c r="F2180" t="inlineStr">
+        <is>
+          <t>3-15</t>
+        </is>
+      </c>
+      <c r="G2180" t="inlineStr">
+        <is>
+          <t>3-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="C2181" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2181" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2181" t="inlineStr">
+        <is>
+          <t>O'Donnell Park, Letterkenny</t>
+        </is>
+      </c>
+      <c r="F2181" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+      <c r="G2181" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2182" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2182" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2182" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2182" t="inlineStr">
+        <is>
+          <t>Technological University Dublin Blanchardstown Campus</t>
+        </is>
+      </c>
+      <c r="F2182" t="inlineStr">
+        <is>
+          <t>3-15</t>
+        </is>
+      </c>
+      <c r="G2182" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="C2183" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2183" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2183" t="inlineStr">
+        <is>
+          <t>Templemore</t>
+        </is>
+      </c>
+      <c r="F2183" t="inlineStr">
+        <is>
+          <t>1-9</t>
+        </is>
+      </c>
+      <c r="G2183" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2184" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2184" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2184" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2184" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park, Portlaoise</t>
+        </is>
+      </c>
+      <c r="F2184" t="inlineStr">
+        <is>
+          <t>3-13</t>
+        </is>
+      </c>
+      <c r="G2184" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2185" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2185" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2185" t="inlineStr">
+        <is>
+          <t>Weavers Fields</t>
+        </is>
+      </c>
+      <c r="F2185" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+      <c r="G2185" t="inlineStr">
+        <is>
+          <t>1-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2186" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2186" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2186" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2186" t="inlineStr">
+        <is>
+          <t>McKenna Park, Ballycran</t>
+        </is>
+      </c>
+      <c r="F2186" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+      <c r="G2186" t="inlineStr">
+        <is>
+          <t>3-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="C2187" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2187" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2187" t="inlineStr">
+        <is>
+          <t>TEG Cusack Park, Westmeath</t>
+        </is>
+      </c>
+      <c r="F2187" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+      <c r="G2187" t="inlineStr">
+        <is>
+          <t>5-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2188" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2188" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2188" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2188" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Newbridge</t>
+        </is>
+      </c>
+      <c r="F2188" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+      <c r="G2188" t="inlineStr">
+        <is>
+          <t>4-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="C2189" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2189" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2189" t="inlineStr">
+        <is>
+          <t>Chadwicks Wexford Park</t>
+        </is>
+      </c>
+      <c r="F2189" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+      <c r="G2189" t="inlineStr">
+        <is>
+          <t>2-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2190" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2190" t="inlineStr">
+        <is>
+          <t>Lancashire</t>
+        </is>
+      </c>
+      <c r="D2190" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2190" t="inlineStr">
+        <is>
+          <t>Inniskeen</t>
+        </is>
+      </c>
+      <c r="F2190" t="inlineStr">
+        <is>
+          <t>0-28</t>
+        </is>
+      </c>
+      <c r="G2190" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="C2191" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2191" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2191" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2191" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2191" t="inlineStr">
+        <is>
+          <t>3-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2192" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2192" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="D2192" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2192" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2192" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2192" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2193" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2193" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2193" t="inlineStr">
+        <is>
+          <t>Azzurri Walsh Park, Waterford</t>
+        </is>
+      </c>
+      <c r="F2193" t="inlineStr">
+        <is>
+          <t>0-25</t>
+        </is>
+      </c>
+      <c r="G2193" t="inlineStr">
+        <is>
+          <t>1-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2194" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2194" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2194" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2194" t="inlineStr">
+        <is>
+          <t>Thomas Davis, Corrinshego</t>
+        </is>
+      </c>
+      <c r="F2194" t="inlineStr">
+        <is>
+          <t>3-16</t>
+        </is>
+      </c>
+      <c r="G2194" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2195" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C2195" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="D2195" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2195" t="inlineStr">
+        <is>
+          <t>Hastings Insurance MacHale Park, Castlebar</t>
+        </is>
+      </c>
+      <c r="F2195" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+      <c r="G2195" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2196" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2196" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2196" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2196" t="inlineStr">
+        <is>
+          <t>Garvaghey</t>
+        </is>
+      </c>
+      <c r="F2196" t="inlineStr">
+        <is>
+          <t>3-21</t>
+        </is>
+      </c>
+      <c r="G2196" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2197" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2197" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="D2197" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2197" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2197" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+      <c r="G2197" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2198" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="C2198" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2198" t="inlineStr">
+        <is>
+          <t>09/05/2026</t>
+        </is>
+      </c>
+      <c r="E2198" t="inlineStr">
+        <is>
+          <t>Chadwicks Wexford Park</t>
+        </is>
+      </c>
+      <c r="F2198" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+      <c r="G2198" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-10
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2198"/>
+  <dimension ref="A1:G2209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78134,6 +78134,413 @@
         </is>
       </c>
     </row>
+    <row r="2199">
+      <c r="A2199" t="inlineStr">
+        <is>
+          <t>Connacht GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2199" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2199" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2199" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2199" t="inlineStr">
+        <is>
+          <t>King &amp; Moffatt Dr. Hyde Park</t>
+        </is>
+      </c>
+      <c r="F2199" t="inlineStr">
+        <is>
+          <t>3-21</t>
+        </is>
+      </c>
+      <c r="G2199" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" t="inlineStr">
+        <is>
+          <t>Dalata Hotel Group GAA Football All-Ireland U20B Championship</t>
+        </is>
+      </c>
+      <c r="B2200" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2200" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2200" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2200" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2200" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2200" t="inlineStr">
+        <is>
+          <t>0-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2201" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="C2201" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2201" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2201" t="inlineStr">
+        <is>
+          <t>UPMC Nowlan Park, Kilkenny</t>
+        </is>
+      </c>
+      <c r="F2201" t="inlineStr">
+        <is>
+          <t>1-6</t>
+        </is>
+      </c>
+      <c r="G2201" t="inlineStr">
+        <is>
+          <t>5-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2202" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2202" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="D2202" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2202" t="inlineStr">
+        <is>
+          <t>McGovern Park, Ruislip</t>
+        </is>
+      </c>
+      <c r="F2202" t="inlineStr">
+        <is>
+          <t>4-9</t>
+        </is>
+      </c>
+      <c r="G2202" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2203" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2203" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="D2203" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2203" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park, Tullamore</t>
+        </is>
+      </c>
+      <c r="F2203" t="inlineStr">
+        <is>
+          <t>0-24</t>
+        </is>
+      </c>
+      <c r="G2203" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" t="inlineStr">
+        <is>
+          <t>Munster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2204" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2204" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2204" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2204" t="inlineStr">
+        <is>
+          <t>Fitzgerald Stadium, Killarney</t>
+        </is>
+      </c>
+      <c r="F2204" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G2204" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2205" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2205" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2205" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2205" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2205" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+      <c r="G2205" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2206" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2206" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="D2206" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2206" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park, Carlow</t>
+        </is>
+      </c>
+      <c r="F2206" t="inlineStr">
+        <is>
+          <t>2-26</t>
+        </is>
+      </c>
+      <c r="G2206" t="inlineStr">
+        <is>
+          <t>6-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2207" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2207" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2207" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2207" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park, Portlaoise</t>
+        </is>
+      </c>
+      <c r="F2207" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G2207" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2208" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2208" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D2208" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2208" t="inlineStr">
+        <is>
+          <t>Cappoquin Logistics Fraher Field</t>
+        </is>
+      </c>
+      <c r="F2208" t="inlineStr">
+        <is>
+          <t>0-10</t>
+        </is>
+      </c>
+      <c r="G2208" t="inlineStr">
+        <is>
+          <t>5-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2209" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2209" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2209" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="E2209" t="inlineStr">
+        <is>
+          <t>Brewster Park, Enniskillen</t>
+        </is>
+      </c>
+      <c r="F2209" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+      <c r="G2209" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-13
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2209"/>
+  <dimension ref="A1:G2212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78541,6 +78541,117 @@
         </is>
       </c>
     </row>
+    <row r="2210">
+      <c r="A2210" t="inlineStr">
+        <is>
+          <t>Dalata Hotel Group GAA Football All-Ireland U20 Championship</t>
+        </is>
+      </c>
+      <c r="B2210" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2210" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2210" t="inlineStr">
+        <is>
+          <t>13/05/2026</t>
+        </is>
+      </c>
+      <c r="E2210" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2210" t="inlineStr">
+        <is>
+          <t>3-17</t>
+        </is>
+      </c>
+      <c r="G2210" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" t="inlineStr">
+        <is>
+          <t>Dalata Hotel Group GAA Football All-Ireland U20 Championship</t>
+        </is>
+      </c>
+      <c r="B2211" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2211" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2211" t="inlineStr">
+        <is>
+          <t>13/05/2026</t>
+        </is>
+      </c>
+      <c r="E2211" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2211" t="inlineStr">
+        <is>
+          <t>0-13</t>
+        </is>
+      </c>
+      <c r="G2211" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" t="inlineStr">
+        <is>
+          <t>Dalata Hotel Group GAA Football All-Ireland U20B Championship</t>
+        </is>
+      </c>
+      <c r="B2212" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2212" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2212" t="inlineStr">
+        <is>
+          <t>13/05/2026</t>
+        </is>
+      </c>
+      <c r="E2212" t="inlineStr">
+        <is>
+          <t>Abbottstown - GAA Centre of Excellence</t>
+        </is>
+      </c>
+      <c r="F2212" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+      <c r="G2212" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-15
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2212"/>
+  <dimension ref="A1:G2213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78652,6 +78652,43 @@
         </is>
       </c>
     </row>
+    <row r="2213">
+      <c r="A2213" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2213" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2213" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D2213" t="inlineStr">
+        <is>
+          <t>15/05/2026</t>
+        </is>
+      </c>
+      <c r="E2213" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2213" t="inlineStr">
+        <is>
+          <t>3-18</t>
+        </is>
+      </c>
+      <c r="G2213" t="inlineStr">
+        <is>
+          <t>0-12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-16
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2213"/>
+  <dimension ref="A1:G2232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78689,6 +78689,709 @@
         </is>
       </c>
     </row>
+    <row r="2214">
+      <c r="A2214" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2214" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2214" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2214" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2214" t="inlineStr">
+        <is>
+          <t>Find Insurance Celtic Park, Derry</t>
+        </is>
+      </c>
+      <c r="F2214" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+      <c r="G2214" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2215" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="C2215" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2215" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2215" t="inlineStr">
+        <is>
+          <t>O'Donnell Park, Letterkenny</t>
+        </is>
+      </c>
+      <c r="F2215" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+      <c r="G2215" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2216" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2216" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2216" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2216" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2216" t="inlineStr">
+        <is>
+          <t>3-12</t>
+        </is>
+      </c>
+      <c r="G2216" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2217" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="C2217" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2217" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2217" t="inlineStr">
+        <is>
+          <t>Glennon Brother's Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2217" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+      <c r="G2217" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2218" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2218" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2218" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2218" t="inlineStr">
+        <is>
+          <t>Inniskeen</t>
+        </is>
+      </c>
+      <c r="F2218" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+      <c r="G2218" t="inlineStr">
+        <is>
+          <t>2-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2219" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2219" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D2219" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2219" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park, Carlow</t>
+        </is>
+      </c>
+      <c r="F2219" t="inlineStr">
+        <is>
+          <t>5-27</t>
+        </is>
+      </c>
+      <c r="G2219" t="inlineStr">
+        <is>
+          <t>0-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2220" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2220" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2220" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2220" t="inlineStr">
+        <is>
+          <t>Corrigan Park</t>
+        </is>
+      </c>
+      <c r="F2220" t="inlineStr">
+        <is>
+          <t>2-29</t>
+        </is>
+      </c>
+      <c r="G2220" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2221" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2221" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2221" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2221" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park, Portlaoise</t>
+        </is>
+      </c>
+      <c r="F2221" t="inlineStr">
+        <is>
+          <t>4-28</t>
+        </is>
+      </c>
+      <c r="G2221" t="inlineStr">
+        <is>
+          <t>0-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2222" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2222" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2222" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2222" t="inlineStr">
+        <is>
+          <t>Pearse Stadium, Salthill</t>
+        </is>
+      </c>
+      <c r="F2222" t="inlineStr">
+        <is>
+          <t>0-21</t>
+        </is>
+      </c>
+      <c r="G2222" t="inlineStr">
+        <is>
+          <t>3-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2223" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="C2223" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="D2223" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2223" t="inlineStr">
+        <is>
+          <t>UPMC Nowlan Park</t>
+        </is>
+      </c>
+      <c r="F2223" t="inlineStr">
+        <is>
+          <t>4-25</t>
+        </is>
+      </c>
+      <c r="G2223" t="inlineStr">
+        <is>
+          <t>0-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2224" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2224" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2224" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2224" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park, Tullamore</t>
+        </is>
+      </c>
+      <c r="F2224" t="inlineStr">
+        <is>
+          <t>2-21</t>
+        </is>
+      </c>
+      <c r="G2224" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2225" t="inlineStr">
+        <is>
+          <t>Lancashire</t>
+        </is>
+      </c>
+      <c r="C2225" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="D2225" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2225" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2225" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+      <c r="G2225" t="inlineStr">
+        <is>
+          <t>6-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2226" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2226" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2226" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2226" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2226" t="inlineStr">
+        <is>
+          <t>1-23</t>
+        </is>
+      </c>
+      <c r="G2226" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2227" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="C2227" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="D2227" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2227" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2227" t="inlineStr">
+        <is>
+          <t>4-16</t>
+        </is>
+      </c>
+      <c r="G2227" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2228" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="C2228" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="D2228" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2228" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2228" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+      <c r="G2228" t="inlineStr">
+        <is>
+          <t>1-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2229" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2229" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2229" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2229" t="inlineStr">
+        <is>
+          <t>Dowdallshill, Dundalk</t>
+        </is>
+      </c>
+      <c r="F2229" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+      <c r="G2229" t="inlineStr">
+        <is>
+          <t>3-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2230" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2230" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2230" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2230" t="inlineStr">
+        <is>
+          <t>Markievicz Park, Sligo</t>
+        </is>
+      </c>
+      <c r="F2230" t="inlineStr">
+        <is>
+          <t>3-29</t>
+        </is>
+      </c>
+      <c r="G2230" t="inlineStr">
+        <is>
+          <t>2-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2231" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2231" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2231" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2231" t="inlineStr">
+        <is>
+          <t>Garvaghey</t>
+        </is>
+      </c>
+      <c r="F2231" t="inlineStr">
+        <is>
+          <t>8-15</t>
+        </is>
+      </c>
+      <c r="G2231" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2232" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2232" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="D2232" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="E2232" t="inlineStr">
+        <is>
+          <t>Páirc Esler, Newry</t>
+        </is>
+      </c>
+      <c r="F2232" t="inlineStr">
+        <is>
+          <t>1-27</t>
+        </is>
+      </c>
+      <c r="G2232" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-17
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2232"/>
+  <dimension ref="A1:G2235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79392,6 +79392,117 @@
         </is>
       </c>
     </row>
+    <row r="2233">
+      <c r="A2233" t="inlineStr">
+        <is>
+          <t>Leinster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2233" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2233" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2233" t="inlineStr">
+        <is>
+          <t>17/05/2026</t>
+        </is>
+      </c>
+      <c r="E2233" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2233" t="inlineStr">
+        <is>
+          <t>0-26</t>
+        </is>
+      </c>
+      <c r="G2233" t="inlineStr">
+        <is>
+          <t>2-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2234" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2234" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="D2234" t="inlineStr">
+        <is>
+          <t>17/05/2026</t>
+        </is>
+      </c>
+      <c r="E2234" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2234" t="inlineStr">
+        <is>
+          <t>2-29</t>
+        </is>
+      </c>
+      <c r="G2234" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" t="inlineStr">
+        <is>
+          <t>Ulster GAA Football Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2235" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2235" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2235" t="inlineStr">
+        <is>
+          <t>17/05/2026</t>
+        </is>
+      </c>
+      <c r="E2235" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2235" t="inlineStr">
+        <is>
+          <t>0-25</t>
+        </is>
+      </c>
+      <c r="G2235" t="inlineStr">
+        <is>
+          <t>2-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-25
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2235"/>
+  <dimension ref="A1:G2265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -79503,6 +79503,1116 @@
         </is>
       </c>
     </row>
+    <row r="2236">
+      <c r="A2236" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2236" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2236" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2236" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2236" t="inlineStr">
+        <is>
+          <t>Fitzgerald Stadium, Killarney</t>
+        </is>
+      </c>
+      <c r="F2236" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+      <c r="G2236" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2237" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2237" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2237" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2237" t="inlineStr">
+        <is>
+          <t>Páirc Uí Rinn</t>
+        </is>
+      </c>
+      <c r="F2237" t="inlineStr">
+        <is>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="G2237" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2238" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2238" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="D2238" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2238" t="inlineStr">
+        <is>
+          <t>Pearse Stadium, Salthill</t>
+        </is>
+      </c>
+      <c r="F2238" t="inlineStr">
+        <is>
+          <t>3-21</t>
+        </is>
+      </c>
+      <c r="G2238" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" t="inlineStr">
+        <is>
+          <t>Dalata Hotel Group GAA Football All-Ireland U20B Championship</t>
+        </is>
+      </c>
+      <c r="B2239" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2239" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="D2239" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2239" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park, Tullamore</t>
+        </is>
+      </c>
+      <c r="F2239" t="inlineStr">
+        <is>
+          <t>0-8</t>
+        </is>
+      </c>
+      <c r="G2239" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Hurling Championship</t>
+        </is>
+      </c>
+      <c r="B2240" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2240" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="D2240" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2240" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2240" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+      <c r="G2240" t="inlineStr">
+        <is>
+          <t>3-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Hurling Championship</t>
+        </is>
+      </c>
+      <c r="B2241" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2241" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2241" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2241" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2241" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+      <c r="G2241" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2242" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2242" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2242" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2242" t="inlineStr">
+        <is>
+          <t>St Peregrine's, Dublin</t>
+        </is>
+      </c>
+      <c r="F2242" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+      <c r="G2242" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2243" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2243" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2243" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2243" t="inlineStr">
+        <is>
+          <t>Netwatch Cullen Park, Carlow</t>
+        </is>
+      </c>
+      <c r="F2243" t="inlineStr">
+        <is>
+          <t>1-9</t>
+        </is>
+      </c>
+      <c r="G2243" t="inlineStr">
+        <is>
+          <t>0-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2244" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="C2244" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="D2244" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2244" t="inlineStr">
+        <is>
+          <t>Kilcoyne Park, Tubbercurry</t>
+        </is>
+      </c>
+      <c r="F2244" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+      <c r="G2244" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2245" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2245" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2245" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2245" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park, Tullamore</t>
+        </is>
+      </c>
+      <c r="F2245" t="inlineStr">
+        <is>
+          <t>4-22</t>
+        </is>
+      </c>
+      <c r="G2245" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2246" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2246" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2246" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2246" t="inlineStr">
+        <is>
+          <t>Kinnegad</t>
+        </is>
+      </c>
+      <c r="F2246" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+      <c r="G2246" t="inlineStr">
+        <is>
+          <t>5-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2247" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2247" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2247" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2247" t="inlineStr">
+        <is>
+          <t>Corduff</t>
+        </is>
+      </c>
+      <c r="F2247" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="G2247" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2248" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2248" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2248" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2248" t="inlineStr">
+        <is>
+          <t>McGovern Park, Ruislip</t>
+        </is>
+      </c>
+      <c r="F2248" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+      <c r="G2248" t="inlineStr">
+        <is>
+          <t>1-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2249" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2249" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2249" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2249" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park, Tullamore</t>
+        </is>
+      </c>
+      <c r="F2249" t="inlineStr">
+        <is>
+          <t>3-22</t>
+        </is>
+      </c>
+      <c r="G2249" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2250" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2250" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2250" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2250" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2250" t="inlineStr">
+        <is>
+          <t>4-17</t>
+        </is>
+      </c>
+      <c r="G2250" t="inlineStr">
+        <is>
+          <t>2-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2251" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2251" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2251" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2251" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2251" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2251" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2252" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2252" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2252" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="E2252" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2252" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+      <c r="G2252" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2253" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2253" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2253" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2253" t="inlineStr">
+        <is>
+          <t>King &amp; Moffatt Dr. Hyde Park</t>
+        </is>
+      </c>
+      <c r="F2253" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+      <c r="G2253" t="inlineStr">
+        <is>
+          <t>3-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2254" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2254" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="D2254" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2254" t="inlineStr">
+        <is>
+          <t>Parnell Park, Dublin</t>
+        </is>
+      </c>
+      <c r="F2254" t="inlineStr">
+        <is>
+          <t>1-26</t>
+        </is>
+      </c>
+      <c r="G2254" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2255" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2255" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="D2255" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2255" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Newbridge</t>
+        </is>
+      </c>
+      <c r="F2255" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+      <c r="G2255" t="inlineStr">
+        <is>
+          <t>1-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2256" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="C2256" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2256" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2256" t="inlineStr">
+        <is>
+          <t>Chadwicks Wexford Park</t>
+        </is>
+      </c>
+      <c r="F2256" t="inlineStr">
+        <is>
+          <t>3-20</t>
+        </is>
+      </c>
+      <c r="G2256" t="inlineStr">
+        <is>
+          <t>2-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2257" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2257" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="D2257" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2257" t="inlineStr">
+        <is>
+          <t>SuperValu Páirc Uí Chaoimh, Cork</t>
+        </is>
+      </c>
+      <c r="F2257" t="inlineStr">
+        <is>
+          <t>1-30</t>
+        </is>
+      </c>
+      <c r="G2257" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2258" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2258" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2258" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2258" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2258" t="inlineStr">
+        <is>
+          <t>5-27</t>
+        </is>
+      </c>
+      <c r="G2258" t="inlineStr">
+        <is>
+          <t>0-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2259" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C2259" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D2259" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2259" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2259" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2259" t="inlineStr">
+        <is>
+          <t>4-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2260" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2260" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="D2260" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2260" t="inlineStr">
+        <is>
+          <t>Corrigan Park</t>
+        </is>
+      </c>
+      <c r="F2260" t="inlineStr">
+        <is>
+          <t>3-26</t>
+        </is>
+      </c>
+      <c r="G2260" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2261" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2261" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2261" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2261" t="inlineStr">
+        <is>
+          <t>McKenna Park, Ballycran</t>
+        </is>
+      </c>
+      <c r="F2261" t="inlineStr">
+        <is>
+          <t>1-28</t>
+        </is>
+      </c>
+      <c r="G2261" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2262" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2262" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2262" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2262" t="inlineStr">
+        <is>
+          <t>McGovern Park, Ruislip</t>
+        </is>
+      </c>
+      <c r="F2262" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+      <c r="G2262" t="inlineStr">
+        <is>
+          <t>1-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2263" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2263" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2263" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2263" t="inlineStr">
+        <is>
+          <t>Brewster Park, Enniskillen</t>
+        </is>
+      </c>
+      <c r="F2263" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2263" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2264" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2264" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2264" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2264" t="inlineStr">
+        <is>
+          <t>Corrigan Park</t>
+        </is>
+      </c>
+      <c r="F2264" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+      <c r="G2264" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2265" t="inlineStr">
+        <is>
+          <t>Waterford</t>
+        </is>
+      </c>
+      <c r="C2265" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="D2265" t="inlineStr">
+        <is>
+          <t>24/05/2026</t>
+        </is>
+      </c>
+      <c r="E2265" t="inlineStr">
+        <is>
+          <t>Cappoquin Logistics Fraher Field</t>
+        </is>
+      </c>
+      <c r="F2265" t="inlineStr">
+        <is>
+          <t>3-12</t>
+        </is>
+      </c>
+      <c r="G2265" t="inlineStr">
+        <is>
+          <t>0-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-29
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2265"/>
+  <dimension ref="A1:G2266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80613,6 +80613,43 @@
         </is>
       </c>
     </row>
+    <row r="2266">
+      <c r="A2266" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2266" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2266" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="D2266" t="inlineStr">
+        <is>
+          <t>29/05/2026</t>
+        </is>
+      </c>
+      <c r="E2266" t="inlineStr">
+        <is>
+          <t>Ballinlough GAA Club</t>
+        </is>
+      </c>
+      <c r="F2266" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+      <c r="G2266" t="inlineStr">
+        <is>
+          <t>2-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-30
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2266"/>
+  <dimension ref="A1:G2276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80650,6 +80650,376 @@
         </is>
       </c>
     </row>
+    <row r="2267">
+      <c r="A2267" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2267" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="C2267" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="D2267" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2267" t="inlineStr">
+        <is>
+          <t>TEG Cusack Park, Westmeath</t>
+        </is>
+      </c>
+      <c r="F2267" t="inlineStr">
+        <is>
+          <t>1-31</t>
+        </is>
+      </c>
+      <c r="G2267" t="inlineStr">
+        <is>
+          <t>3-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2268" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="C2268" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="D2268" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2268" t="inlineStr">
+        <is>
+          <t>BOX-IT Athletic Grounds, Armagh</t>
+        </is>
+      </c>
+      <c r="F2268" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2268" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" t="inlineStr">
+        <is>
+          <t>Christy Ring Cup</t>
+        </is>
+      </c>
+      <c r="B2269" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2269" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2269" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2269" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2269" t="inlineStr">
+        <is>
+          <t>3-24</t>
+        </is>
+      </c>
+      <c r="G2269" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" t="inlineStr">
+        <is>
+          <t>Nickey Rackard Cup</t>
+        </is>
+      </c>
+      <c r="B2270" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C2270" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2270" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2270" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2270" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+      <c r="G2270" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" t="inlineStr">
+        <is>
+          <t>Dalata Hotel Group GAA Football All-Ireland U20 Championship</t>
+        </is>
+      </c>
+      <c r="B2271" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2271" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2271" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2271" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2271" t="inlineStr">
+        <is>
+          <t>0-21</t>
+        </is>
+      </c>
+      <c r="G2271" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Hurling Championship</t>
+        </is>
+      </c>
+      <c r="B2272" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2272" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="D2272" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2272" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2272" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+      <c r="G2272" t="inlineStr">
+        <is>
+          <t>0-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Hurling Championship</t>
+        </is>
+      </c>
+      <c r="B2273" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="C2273" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2273" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2273" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2273" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+      <c r="G2273" t="inlineStr">
+        <is>
+          <t>2-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Tier 3 Championship (Seamus Heaney Cup)</t>
+        </is>
+      </c>
+      <c r="B2274" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2274" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2274" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2274" t="inlineStr">
+        <is>
+          <t>Inniskeen</t>
+        </is>
+      </c>
+      <c r="F2274" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2274" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2275" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2275" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2275" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2275" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2275" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+      <c r="G2275" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2276" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2276" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="D2276" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E2276" t="inlineStr">
+        <is>
+          <t>Glennon Brothers Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2276" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+      <c r="G2276" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-05-31
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2276"/>
+  <dimension ref="A1:G2280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81020,6 +81020,154 @@
         </is>
       </c>
     </row>
+    <row r="2277">
+      <c r="A2277" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2277" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2277" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2277" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="E2277" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2277" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+      <c r="G2277" t="inlineStr">
+        <is>
+          <t>4-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2278" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2278" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2278" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="E2278" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2278" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2278" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" t="inlineStr">
+        <is>
+          <t>Lory Meagher Cup</t>
+        </is>
+      </c>
+      <c r="B2279" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2279" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="D2279" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="E2279" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2279" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+      <c r="G2279" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" t="inlineStr">
+        <is>
+          <t>Fulfil GAA Hurling All-Ireland U20 Championship</t>
+        </is>
+      </c>
+      <c r="B2280" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2280" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2280" t="inlineStr">
+        <is>
+          <t>31/05/2026</t>
+        </is>
+      </c>
+      <c r="E2280" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2280" t="inlineStr">
+        <is>
+          <t>4-20</t>
+        </is>
+      </c>
+      <c r="G2280" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-06
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2280"/>
+  <dimension ref="A1:G2293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81168,6 +81168,487 @@
         </is>
       </c>
     </row>
+    <row r="2281">
+      <c r="A2281" t="inlineStr">
+        <is>
+          <t>Leinster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2281" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2281" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2281" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2281" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2281" t="inlineStr">
+        <is>
+          <t>4-15</t>
+        </is>
+      </c>
+      <c r="G2281" t="inlineStr">
+        <is>
+          <t>4-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2282" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2282" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2282" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2282" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2282" t="inlineStr">
+        <is>
+          <t>3-19</t>
+        </is>
+      </c>
+      <c r="G2282" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2283" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2283" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2283" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2283" t="inlineStr">
+        <is>
+          <t>Ashbourne</t>
+        </is>
+      </c>
+      <c r="F2283" t="inlineStr">
+        <is>
+          <t>3-17</t>
+        </is>
+      </c>
+      <c r="G2283" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2284" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2284" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2284" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2284" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2284" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+      <c r="G2284" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2285" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="C2285" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="D2285" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2285" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2285" t="inlineStr">
+        <is>
+          <t>1-9</t>
+        </is>
+      </c>
+      <c r="G2285" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2286" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2286" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="D2286" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2286" t="inlineStr">
+        <is>
+          <t>Cullyhanna</t>
+        </is>
+      </c>
+      <c r="F2286" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+      <c r="G2286" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2287" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2287" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2287" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2287" t="inlineStr">
+        <is>
+          <t>Scotstown</t>
+        </is>
+      </c>
+      <c r="F2287" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+      <c r="G2287" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" t="inlineStr">
+        <is>
+          <t>Joe McDonagh Cup</t>
+        </is>
+      </c>
+      <c r="B2288" t="inlineStr">
+        <is>
+          <t>Carlow</t>
+        </is>
+      </c>
+      <c r="C2288" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="D2288" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2288" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2288" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2288" t="inlineStr">
+        <is>
+          <t>1-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2289" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2289" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="D2289" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2289" t="inlineStr">
+        <is>
+          <t>McGovern Park, Ruislip</t>
+        </is>
+      </c>
+      <c r="F2289" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+      <c r="G2289" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2290" t="inlineStr">
+        <is>
+          <t>Leitrim</t>
+        </is>
+      </c>
+      <c r="C2290" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2290" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2290" t="inlineStr">
+        <is>
+          <t>Heartland Credit Union Páirc Seán MacDiarmada</t>
+        </is>
+      </c>
+      <c r="F2290" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+      <c r="G2290" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2291" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="C2291" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2291" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2291" t="inlineStr">
+        <is>
+          <t>Echelon Park, Aughrim</t>
+        </is>
+      </c>
+      <c r="F2291" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+      <c r="G2291" t="inlineStr">
+        <is>
+          <t>0-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2292" t="inlineStr">
+        <is>
+          <t>Longford</t>
+        </is>
+      </c>
+      <c r="C2292" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2292" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2292" t="inlineStr">
+        <is>
+          <t>Glennon Brother's Pearse Park</t>
+        </is>
+      </c>
+      <c r="F2292" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2292" t="inlineStr">
+        <is>
+          <t>4-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2293" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2293" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="D2293" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2293" t="inlineStr">
+        <is>
+          <t>Brewster Park, Enniskillen</t>
+        </is>
+      </c>
+      <c r="F2293" t="inlineStr">
+        <is>
+          <t>3-27</t>
+        </is>
+      </c>
+      <c r="G2293" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-07
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2293"/>
+  <dimension ref="A1:G2294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81649,6 +81649,43 @@
         </is>
       </c>
     </row>
+    <row r="2294">
+      <c r="A2294" t="inlineStr">
+        <is>
+          <t>Munster GAA Hurling Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2294" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2294" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2294" t="inlineStr">
+        <is>
+          <t>07/06/2026</t>
+        </is>
+      </c>
+      <c r="E2294" t="inlineStr">
+        <is>
+          <t>SuperValu Páirc Uí Chaoimh, Cork</t>
+        </is>
+      </c>
+      <c r="F2294" t="inlineStr">
+        <is>
+          <t>2-17</t>
+        </is>
+      </c>
+      <c r="G2294" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-13
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2294"/>
+  <dimension ref="A1:G2305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81686,6 +81686,413 @@
         </is>
       </c>
     </row>
+    <row r="2295">
+      <c r="A2295" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2295" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="C2295" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2295" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2295" t="inlineStr">
+        <is>
+          <t>MacCumhaill Park, Ballybofey</t>
+        </is>
+      </c>
+      <c r="F2295" t="inlineStr">
+        <is>
+          <t>1-13</t>
+        </is>
+      </c>
+      <c r="G2295" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2296" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2296" t="inlineStr">
+        <is>
+          <t>Roscommon</t>
+        </is>
+      </c>
+      <c r="D2296" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2296" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2296" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+      <c r="G2296" t="inlineStr">
+        <is>
+          <t>0-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2297" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2297" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2297" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2297" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Park, Newbridge</t>
+        </is>
+      </c>
+      <c r="F2297" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+      <c r="G2297" t="inlineStr">
+        <is>
+          <t>3-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2298" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="C2298" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2298" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2298" t="inlineStr">
+        <is>
+          <t>Find Insurance Celtic Park, Derry</t>
+        </is>
+      </c>
+      <c r="F2298" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+      <c r="G2298" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Hurling Championship</t>
+        </is>
+      </c>
+      <c r="B2299" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="C2299" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="D2299" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2299" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2299" t="inlineStr">
+        <is>
+          <t>5-18</t>
+        </is>
+      </c>
+      <c r="G2299" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Hurling Championship</t>
+        </is>
+      </c>
+      <c r="B2300" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2300" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2300" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2300" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Páirc Chíosóg, Ennis</t>
+        </is>
+      </c>
+      <c r="F2300" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2300" t="inlineStr">
+        <is>
+          <t>1-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Tier 2 Championship (Paul McGirr Cup)</t>
+        </is>
+      </c>
+      <c r="B2301" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="C2301" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="D2301" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2301" t="inlineStr">
+        <is>
+          <t>BOX-IT Athletic Grounds, Armagh</t>
+        </is>
+      </c>
+      <c r="F2301" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2301" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2302" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2302" t="inlineStr">
+        <is>
+          <t>Wexford</t>
+        </is>
+      </c>
+      <c r="D2302" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2302" t="inlineStr">
+        <is>
+          <t>Glenisk O'Connor Park, Tullamore</t>
+        </is>
+      </c>
+      <c r="F2302" t="inlineStr">
+        <is>
+          <t>1-22</t>
+        </is>
+      </c>
+      <c r="G2302" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2303" t="inlineStr">
+        <is>
+          <t>Antrim</t>
+        </is>
+      </c>
+      <c r="C2303" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2303" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2303" t="inlineStr">
+        <is>
+          <t>Corrigan Park</t>
+        </is>
+      </c>
+      <c r="F2303" t="inlineStr">
+        <is>
+          <t>3-15</t>
+        </is>
+      </c>
+      <c r="G2303" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2304" t="inlineStr">
+        <is>
+          <t>Laois</t>
+        </is>
+      </c>
+      <c r="C2304" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="D2304" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2304" t="inlineStr">
+        <is>
+          <t>Laois Hire O'Moore Park, Portlaoise</t>
+        </is>
+      </c>
+      <c r="F2304" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+      <c r="G2304" t="inlineStr">
+        <is>
+          <t>2-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2305" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="C2305" t="inlineStr">
+        <is>
+          <t>Sligo</t>
+        </is>
+      </c>
+      <c r="D2305" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="E2305" t="inlineStr">
+        <is>
+          <t>Brewster Park, Enniskillen</t>
+        </is>
+      </c>
+      <c r="F2305" t="inlineStr">
+        <is>
+          <t>2-25</t>
+        </is>
+      </c>
+      <c r="G2305" t="inlineStr">
+        <is>
+          <t>0-9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-14
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2305"/>
+  <dimension ref="A1:G2309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82093,6 +82093,154 @@
         </is>
       </c>
     </row>
+    <row r="2306">
+      <c r="A2306" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2306" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2306" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2306" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="E2306" t="inlineStr">
+        <is>
+          <t>Páirc Grattan, Inniskeen</t>
+        </is>
+      </c>
+      <c r="F2306" t="inlineStr">
+        <is>
+          <t>2-20</t>
+        </is>
+      </c>
+      <c r="G2306" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2307" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2307" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2307" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="E2307" t="inlineStr">
+        <is>
+          <t>Pearse Stadium, Salthill</t>
+        </is>
+      </c>
+      <c r="F2307" t="inlineStr">
+        <is>
+          <t>3-21</t>
+        </is>
+      </c>
+      <c r="G2307" t="inlineStr">
+        <is>
+          <t>2-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2308" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2308" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2308" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="E2308" t="inlineStr">
+        <is>
+          <t>O'Neills Healy Park, Omagh</t>
+        </is>
+      </c>
+      <c r="F2308" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+      <c r="G2308" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="A2309" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2309" t="inlineStr">
+        <is>
+          <t>Cavan</t>
+        </is>
+      </c>
+      <c r="C2309" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2309" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="E2309" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2309" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+      <c r="G2309" t="inlineStr">
+        <is>
+          <t>1-24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-19
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2309"/>
+  <dimension ref="A1:G2310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82241,6 +82241,43 @@
         </is>
       </c>
     </row>
+    <row r="2310">
+      <c r="A2310" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2310" t="inlineStr">
+        <is>
+          <t>Kildare</t>
+        </is>
+      </c>
+      <c r="C2310" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2310" t="inlineStr">
+        <is>
+          <t>19/06/2026</t>
+        </is>
+      </c>
+      <c r="E2310" t="inlineStr">
+        <is>
+          <t>Kingspan Breffni, Cavan</t>
+        </is>
+      </c>
+      <c r="F2310" t="inlineStr">
+        <is>
+          <t>1-12</t>
+        </is>
+      </c>
+      <c r="G2310" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-20
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2310"/>
+  <dimension ref="A1:G2316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82278,6 +82278,228 @@
         </is>
       </c>
     </row>
+    <row r="2311">
+      <c r="A2311" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2311" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2311" t="inlineStr">
+        <is>
+          <t>Armagh</t>
+        </is>
+      </c>
+      <c r="D2311" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E2311" t="inlineStr">
+        <is>
+          <t>Fitzgerald Stadium, Killarney</t>
+        </is>
+      </c>
+      <c r="F2311" t="inlineStr">
+        <is>
+          <t>4-18</t>
+        </is>
+      </c>
+      <c r="G2311" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2312" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C2312" t="inlineStr">
+        <is>
+          <t>Meath</t>
+        </is>
+      </c>
+      <c r="D2312" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E2312" t="inlineStr">
+        <is>
+          <t>Hastings Insurance MacHale Park, Castlebar</t>
+        </is>
+      </c>
+      <c r="F2312" t="inlineStr">
+        <is>
+          <t>0-22</t>
+        </is>
+      </c>
+      <c r="G2312" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" t="inlineStr">
+        <is>
+          <t>GAA Hurling All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2313" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2313" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="D2313" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E2313" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2313" t="inlineStr">
+        <is>
+          <t>0-29</t>
+        </is>
+      </c>
+      <c r="G2313" t="inlineStr">
+        <is>
+          <t>0-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2314" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2314" t="inlineStr">
+        <is>
+          <t>Derry</t>
+        </is>
+      </c>
+      <c r="D2314" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E2314" t="inlineStr">
+        <is>
+          <t>Parnell Park, Dublin</t>
+        </is>
+      </c>
+      <c r="F2314" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+      <c r="G2314" t="inlineStr">
+        <is>
+          <t>2-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2315" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2315" t="inlineStr">
+        <is>
+          <t>Fermanagh</t>
+        </is>
+      </c>
+      <c r="D2315" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E2315" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2315" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+      <c r="G2315" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="A2316" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2316" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="C2316" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2316" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="E2316" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2316" t="inlineStr">
+        <is>
+          <t>4-15</t>
+        </is>
+      </c>
+      <c r="G2316" t="inlineStr">
+        <is>
+          <t>2-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-21
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2316"/>
+  <dimension ref="A1:G2319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82500,6 +82500,117 @@
         </is>
       </c>
     </row>
+    <row r="2317">
+      <c r="A2317" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2317" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2317" t="inlineStr">
+        <is>
+          <t>Donegal</t>
+        </is>
+      </c>
+      <c r="D2317" t="inlineStr">
+        <is>
+          <t>21/06/2026</t>
+        </is>
+      </c>
+      <c r="E2317" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2317" t="inlineStr">
+        <is>
+          <t>2-26</t>
+        </is>
+      </c>
+      <c r="G2317" t="inlineStr">
+        <is>
+          <t>2-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2318" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2318" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2318" t="inlineStr">
+        <is>
+          <t>21/06/2026</t>
+        </is>
+      </c>
+      <c r="E2318" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2318" t="inlineStr">
+        <is>
+          <t>1-28</t>
+        </is>
+      </c>
+      <c r="G2318" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" t="inlineStr">
+        <is>
+          <t>GAA Hurling All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2319" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2319" t="inlineStr">
+        <is>
+          <t>Offaly</t>
+        </is>
+      </c>
+      <c r="D2319" t="inlineStr">
+        <is>
+          <t>21/06/2026</t>
+        </is>
+      </c>
+      <c r="E2319" t="inlineStr">
+        <is>
+          <t>FBD Semple Stadium, Thurles</t>
+        </is>
+      </c>
+      <c r="F2319" t="inlineStr">
+        <is>
+          <t>6-25</t>
+        </is>
+      </c>
+      <c r="G2319" t="inlineStr">
+        <is>
+          <t>2-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-22
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2319"/>
+  <dimension ref="A1:G2320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82611,6 +82611,43 @@
         </is>
       </c>
     </row>
+    <row r="2320">
+      <c r="A2320" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2320" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="C2320" t="inlineStr">
+        <is>
+          <t>Westmeath</t>
+        </is>
+      </c>
+      <c r="D2320" t="inlineStr">
+        <is>
+          <t>21/06/2026</t>
+        </is>
+      </c>
+      <c r="E2320" t="inlineStr">
+        <is>
+          <t>St. Tiernach's Park, Clones</t>
+        </is>
+      </c>
+      <c r="F2320" t="inlineStr">
+        <is>
+          <t>1-28</t>
+        </is>
+      </c>
+      <c r="G2320" t="inlineStr">
+        <is>
+          <t>2-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-23
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2320"/>
+  <dimension ref="A1:G2321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82648,6 +82648,43 @@
         </is>
       </c>
     </row>
+    <row r="2321">
+      <c r="A2321" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2321" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="C2321" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2321" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="E2321" t="inlineStr">
+        <is>
+          <t>Donaghmore Ashbourne GAA</t>
+        </is>
+      </c>
+      <c r="F2321" t="inlineStr">
+        <is>
+          <t>3-17</t>
+        </is>
+      </c>
+      <c r="G2321" t="inlineStr">
+        <is>
+          <t>0-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-27
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2321"/>
+  <dimension ref="A1:G2324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82685,6 +82685,117 @@
         </is>
       </c>
     </row>
+    <row r="2322">
+      <c r="A2322" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2322" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2322" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2322" t="inlineStr">
+        <is>
+          <t>27/06/2026</t>
+        </is>
+      </c>
+      <c r="E2322" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2322" t="inlineStr">
+        <is>
+          <t>0-18</t>
+        </is>
+      </c>
+      <c r="G2322" t="inlineStr">
+        <is>
+          <t>0-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Hurling Championship</t>
+        </is>
+      </c>
+      <c r="B2323" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="C2323" t="inlineStr">
+        <is>
+          <t>Tipperary</t>
+        </is>
+      </c>
+      <c r="D2323" t="inlineStr">
+        <is>
+          <t>27/06/2026</t>
+        </is>
+      </c>
+      <c r="E2323" t="inlineStr">
+        <is>
+          <t>TUS Gaelic Grounds</t>
+        </is>
+      </c>
+      <c r="F2323" t="inlineStr">
+        <is>
+          <t>2-12</t>
+        </is>
+      </c>
+      <c r="G2323" t="inlineStr">
+        <is>
+          <t>1-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="A2324" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Junior Championship</t>
+        </is>
+      </c>
+      <c r="B2324" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="C2324" t="inlineStr">
+        <is>
+          <t>Kilkenny</t>
+        </is>
+      </c>
+      <c r="D2324" t="inlineStr">
+        <is>
+          <t>27/06/2026</t>
+        </is>
+      </c>
+      <c r="E2324" t="inlineStr">
+        <is>
+          <t>Páirc na hÉireann, Birmingham</t>
+        </is>
+      </c>
+      <c r="F2324" t="inlineStr">
+        <is>
+          <t>1-15</t>
+        </is>
+      </c>
+      <c r="G2324" t="inlineStr">
+        <is>
+          <t>1-10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-06-28
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2324"/>
+  <dimension ref="A1:G2327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82796,6 +82796,117 @@
         </is>
       </c>
     </row>
+    <row r="2325">
+      <c r="A2325" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2325" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2325" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2325" t="inlineStr">
+        <is>
+          <t>27/06/2026</t>
+        </is>
+      </c>
+      <c r="E2325" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2325" t="inlineStr">
+        <is>
+          <t>2-25</t>
+        </is>
+      </c>
+      <c r="G2325" t="inlineStr">
+        <is>
+          <t>0-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="A2326" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2326" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2326" t="inlineStr">
+        <is>
+          <t>Monaghan</t>
+        </is>
+      </c>
+      <c r="D2326" t="inlineStr">
+        <is>
+          <t>28/06/2026</t>
+        </is>
+      </c>
+      <c r="E2326" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2326" t="inlineStr">
+        <is>
+          <t>0-27</t>
+        </is>
+      </c>
+      <c r="G2326" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2327" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2327" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2327" t="inlineStr">
+        <is>
+          <t>28/06/2026</t>
+        </is>
+      </c>
+      <c r="E2327" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2327" t="inlineStr">
+        <is>
+          <t>1-25</t>
+        </is>
+      </c>
+      <c r="G2327" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-07-04
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2327"/>
+  <dimension ref="A1:G2328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82907,6 +82907,43 @@
         </is>
       </c>
     </row>
+    <row r="2328">
+      <c r="A2328" t="inlineStr">
+        <is>
+          <t>GAA Hurling All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2328" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2328" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="D2328" t="inlineStr">
+        <is>
+          <t>04/07/2026</t>
+        </is>
+      </c>
+      <c r="E2328" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2328" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2328" t="inlineStr">
+        <is>
+          <t>2-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-07-05
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2328"/>
+  <dimension ref="A1:G2330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82944,6 +82944,80 @@
         </is>
       </c>
     </row>
+    <row r="2329">
+      <c r="A2329" t="inlineStr">
+        <is>
+          <t>GAA Hurling All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2329" t="inlineStr">
+        <is>
+          <t>Clare</t>
+        </is>
+      </c>
+      <c r="C2329" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2329" t="inlineStr">
+        <is>
+          <t>05/07/2026</t>
+        </is>
+      </c>
+      <c r="E2329" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2329" t="inlineStr">
+        <is>
+          <t>1-19</t>
+        </is>
+      </c>
+      <c r="G2329" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" t="inlineStr">
+        <is>
+          <t>Electric Ireland All-Ireland Minor Football Championship</t>
+        </is>
+      </c>
+      <c r="B2330" t="inlineStr">
+        <is>
+          <t>Cork</t>
+        </is>
+      </c>
+      <c r="C2330" t="inlineStr">
+        <is>
+          <t>Tyrone</t>
+        </is>
+      </c>
+      <c r="D2330" t="inlineStr">
+        <is>
+          <t>05/07/2026</t>
+        </is>
+      </c>
+      <c r="E2330" t="inlineStr">
+        <is>
+          <t>Cedral St Conleth's Newbridge</t>
+        </is>
+      </c>
+      <c r="F2330" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+      <c r="G2330" t="inlineStr">
+        <is>
+          <t>1-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-07-10
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2330"/>
+  <dimension ref="A1:G2332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83018,6 +83018,80 @@
         </is>
       </c>
     </row>
+    <row r="2331">
+      <c r="A2331" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Junior Championship</t>
+        </is>
+      </c>
+      <c r="B2331" t="inlineStr">
+        <is>
+          <t>USGAA</t>
+        </is>
+      </c>
+      <c r="C2331" t="inlineStr">
+        <is>
+          <t>Warwickshire</t>
+        </is>
+      </c>
+      <c r="D2331" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="E2331" t="inlineStr">
+        <is>
+          <t>Abbottstown - GAA Centre of Excellence</t>
+        </is>
+      </c>
+      <c r="F2331" t="inlineStr">
+        <is>
+          <t>2-13</t>
+        </is>
+      </c>
+      <c r="G2331" t="inlineStr">
+        <is>
+          <t>1-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Junior Championship</t>
+        </is>
+      </c>
+      <c r="B2332" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C2332" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D2332" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="E2332" t="inlineStr">
+        <is>
+          <t>Abbottstown - GAA Centre of Excellence</t>
+        </is>
+      </c>
+      <c r="F2332" t="inlineStr">
+        <is>
+          <t>0-13</t>
+        </is>
+      </c>
+      <c r="G2332" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-07-11
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2332"/>
+  <dimension ref="A1:G2334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83092,6 +83092,80 @@
         </is>
       </c>
     </row>
+    <row r="2333">
+      <c r="A2333" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2333" t="inlineStr">
+        <is>
+          <t>Louth</t>
+        </is>
+      </c>
+      <c r="C2333" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2333" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="E2333" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2333" t="inlineStr">
+        <is>
+          <t>0-15</t>
+        </is>
+      </c>
+      <c r="G2333" t="inlineStr">
+        <is>
+          <t>3-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" t="inlineStr">
+        <is>
+          <t>Tailteann Cup</t>
+        </is>
+      </c>
+      <c r="B2334" t="inlineStr">
+        <is>
+          <t>Down</t>
+        </is>
+      </c>
+      <c r="C2334" t="inlineStr">
+        <is>
+          <t>Wicklow</t>
+        </is>
+      </c>
+      <c r="D2334" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="E2334" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2334" t="inlineStr">
+        <is>
+          <t>2-16</t>
+        </is>
+      </c>
+      <c r="G2334" t="inlineStr">
+        <is>
+          <t>1-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-07-12
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2334"/>
+  <dimension ref="A1:G2336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83166,6 +83166,80 @@
         </is>
       </c>
     </row>
+    <row r="2335">
+      <c r="A2335" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2335" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+      <c r="C2335" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="D2335" t="inlineStr">
+        <is>
+          <t>12/07/2026</t>
+        </is>
+      </c>
+      <c r="E2335" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2335" t="inlineStr">
+        <is>
+          <t>0-20</t>
+        </is>
+      </c>
+      <c r="G2335" t="inlineStr">
+        <is>
+          <t>2-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Junior Championship</t>
+        </is>
+      </c>
+      <c r="B2336" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="C2336" t="inlineStr">
+        <is>
+          <t>USGAA</t>
+        </is>
+      </c>
+      <c r="D2336" t="inlineStr">
+        <is>
+          <t>12/07/2026</t>
+        </is>
+      </c>
+      <c r="E2336" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2336" t="inlineStr">
+        <is>
+          <t>5-12</t>
+        </is>
+      </c>
+      <c r="G2336" t="inlineStr">
+        <is>
+          <t>0-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-07-19
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2336"/>
+  <dimension ref="A1:G2337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83240,6 +83240,43 @@
         </is>
       </c>
     </row>
+    <row r="2337">
+      <c r="A2337" t="inlineStr">
+        <is>
+          <t>GAA Hurling All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2337" t="inlineStr">
+        <is>
+          <t>Galway</t>
+        </is>
+      </c>
+      <c r="C2337" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D2337" t="inlineStr">
+        <is>
+          <t>19/07/2026</t>
+        </is>
+      </c>
+      <c r="E2337" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2337" t="inlineStr">
+        <is>
+          <t>1-18</t>
+        </is>
+      </c>
+      <c r="G2337" t="inlineStr">
+        <is>
+          <t>1-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update GAA results for 2026-07-26
</commit_message>
<xml_diff>
--- a/gaa_results.xlsx
+++ b/gaa_results.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2337"/>
+  <dimension ref="A1:G2338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -83277,6 +83277,43 @@
         </is>
       </c>
     </row>
+    <row r="2338">
+      <c r="A2338" t="inlineStr">
+        <is>
+          <t>GAA Football All-Ireland Senior Championship</t>
+        </is>
+      </c>
+      <c r="B2338" t="inlineStr">
+        <is>
+          <t>Kerry</t>
+        </is>
+      </c>
+      <c r="C2338" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="D2338" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="E2338" t="inlineStr">
+        <is>
+          <t>Páirc an Chrócaigh</t>
+        </is>
+      </c>
+      <c r="F2338" t="inlineStr">
+        <is>
+          <t>1-17</t>
+        </is>
+      </c>
+      <c r="G2338" t="inlineStr">
+        <is>
+          <t>1-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>